<commit_message>
[auto-snapshot] 2026-04-17 12:00 | onda-hompage | 23 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_hair/남구_미용실.xlsx
+++ b/naver-place-crawler/results_hair/남구_미용실.xlsx
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>4219</v>
+        <v>4218</v>
       </c>
       <c r="Q2" t="n">
         <v>224</v>
       </c>
       <c r="R2" t="n">
-        <v>4443</v>
+        <v>4442</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -903,13 +903,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>2989</v>
+        <v>2991</v>
       </c>
       <c r="Q5" t="n">
         <v>192</v>
       </c>
       <c r="R5" t="n">
-        <v>3181</v>
+        <v>3183</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -2685,13 +2685,13 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="Q24" t="n">
         <v>35</v>
       </c>
       <c r="R24" t="n">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
@@ -3155,13 +3155,13 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>4524</v>
+        <v>4525</v>
       </c>
       <c r="Q29" t="n">
         <v>56</v>
       </c>
       <c r="R29" t="n">
-        <v>4580</v>
+        <v>4581</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>whitechoco11@naver.com</t>
+          <t>0163891634@naver.com</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ming0104@naver.com</t>
+          <t>gminish@naver.com</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -4008,10 +4008,10 @@
         <v>4372</v>
       </c>
       <c r="Q38" t="n">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="R38" t="n">
-        <v>4846</v>
+        <v>4847</v>
       </c>
       <c r="S38" t="inlineStr">
         <is>
@@ -4862,10 +4862,10 @@
         <v>1472</v>
       </c>
       <c r="Q47" t="n">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="R47" t="n">
-        <v>1673</v>
+        <v>1676</v>
       </c>
       <c r="S47" t="inlineStr">
         <is>
@@ -5141,13 +5141,13 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>2905</v>
+        <v>2906</v>
       </c>
       <c r="Q50" t="n">
         <v>181</v>
       </c>
       <c r="R50" t="n">
-        <v>3086</v>
+        <v>3087</v>
       </c>
       <c r="S50" t="inlineStr">
         <is>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>syn77@naver.com</t>
+          <t>pinkjump010@naver.com</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -6735,13 +6735,13 @@
         </is>
       </c>
       <c r="P67" t="n">
-        <v>2549</v>
+        <v>2547</v>
       </c>
       <c r="Q67" t="n">
         <v>86</v>
       </c>
       <c r="R67" t="n">
-        <v>2635</v>
+        <v>2633</v>
       </c>
       <c r="S67" t="inlineStr">
         <is>
@@ -7243,7 +7243,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>rkddmswl7737@naver.com</t>
+          <t>wlsrud8541@naver.com</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -7275,7 +7275,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-17 16:00 | onda-hompage | 72 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_hair/남구_미용실.xlsx
+++ b/naver-place-crawler/results_hair/남구_미용실.xlsx
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>4218</v>
+        <v>4220</v>
       </c>
       <c r="Q2" t="n">
         <v>224</v>
       </c>
       <c r="R2" t="n">
-        <v>4442</v>
+        <v>4444</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1127,11 +1127,7 @@
           <t>살롱루미에르</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>goto_seoul@naver.com</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
@@ -1369,13 +1365,13 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>11089</v>
+        <v>11091</v>
       </c>
       <c r="Q10" t="n">
         <v>146</v>
       </c>
       <c r="R10" t="n">
-        <v>11235</v>
+        <v>11237</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1409,11 +1405,7 @@
           <t>어뮤트헤어</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>dlsks1022@naver.com</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
@@ -1503,11 +1495,7 @@
           <t>라벨르봄 도화앨리웨이점</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>dnjsrud051@naver.com</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
@@ -1557,13 +1545,13 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="Q12" t="n">
         <v>2</v>
       </c>
       <c r="R12" t="n">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1594,29 +1582,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>누나헤어</t>
+          <t>랑미헤어 인하대역점</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>nuna9664@naver.com</t>
+          <t>rangme_@naver.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0507-1378-4584</t>
+          <t>0507-1489-6557</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 인하로 81 3층 누나헤어</t>
+          <t>인천광역시 미추홀구 소성로 20 2층 202호</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/nuna9664</t>
+          <t>https://www.instagram.com/rang4665</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1631,7 +1619,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1651,13 +1639,13 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>1490</v>
+        <v>1305</v>
       </c>
       <c r="Q13" t="n">
-        <v>21</v>
+        <v>192</v>
       </c>
       <c r="R13" t="n">
-        <v>1511</v>
+        <v>1497</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1666,12 +1654,12 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1864016360</t>
+          <t>1691754307</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1864016360</t>
+          <t>https://m.place.naver.com/place/1691754307</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -1688,34 +1676,34 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>랑미헤어 인하대역점</t>
+          <t>미닝</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>rangme_@naver.com</t>
+          <t>alswjd8914@naver.com</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0507-1489-6557</t>
+          <t>0507-1327-8587</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 소성로 20 2층 202호</t>
+          <t>인천광역시 미추홀구 경인로 372 2층 2070호</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/rang4665</t>
+          <t>http://pf.kakao.com/_tgxbxln</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1736,7 +1724,7 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1745,13 +1733,13 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>1305</v>
+        <v>323</v>
       </c>
       <c r="Q14" t="n">
-        <v>192</v>
+        <v>88</v>
       </c>
       <c r="R14" t="n">
-        <v>1497</v>
+        <v>411</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1760,12 +1748,12 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1691754307</t>
+          <t>1706038921</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1691754307</t>
+          <t>https://m.place.naver.com/place/1706038921</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -1782,34 +1770,34 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>미닝</t>
+          <t>해피꼬헤어</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>alswjd8914@naver.com</t>
+          <t>happy_ggohair@naver.com</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0507-1327-8587</t>
+          <t>0507-1377-1847</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 경인로 372 2층 2070호</t>
+          <t>인천광역시 미추홀구 한나루로489번길 114-4 1층</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>http://pf.kakao.com/_tgxbxln</t>
+          <t>https://blog.naver.com/happy_ggohair</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1819,7 +1807,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1830,7 +1818,7 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1839,13 +1827,13 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>323</v>
+        <v>218</v>
       </c>
       <c r="Q15" t="n">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="R15" t="n">
-        <v>411</v>
+        <v>329</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1854,12 +1842,12 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1706038921</t>
+          <t>1890256512</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1706038921</t>
+          <t>https://m.place.naver.com/place/1890256512</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -1876,29 +1864,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>해피꼬헤어</t>
+          <t>라네프살롱 인하대역점</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>happy_ggohair@naver.com</t>
+          <t>ranefsalon@naver.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0507-1377-1847</t>
+          <t>0507-1448-0603</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 한나루로489번길 114-4 1층</t>
+          <t>인천광역시 미추홀구 독배로 309 노블레스타워 2층 202호 라네프살롱</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/happy_ggohair</t>
+          <t>https://www.instagram.com/ranefsalon_official</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1913,7 +1901,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1933,13 +1921,13 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>218</v>
+        <v>2322</v>
       </c>
       <c r="Q16" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="R16" t="n">
-        <v>329</v>
+        <v>2436</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -1948,12 +1936,12 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1890256512</t>
+          <t>1114490806</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1890256512</t>
+          <t>https://m.place.naver.com/place/1114490806</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
@@ -1970,29 +1958,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>라네프살롱 인하대역점</t>
+          <t>일랑헤어 인하본점</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ranefsalon@naver.com</t>
+          <t>ilranghair11@naver.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0507-1448-0603</t>
+          <t>0507-1429-0212</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 독배로 309 노블레스타워 2층 202호 라네프살롱</t>
+          <t>인천광역시 미추홀구 인하로 73-1</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/ranefsalon_official</t>
+          <t>https://blog.naver.com/ilranghair11</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2007,7 +1995,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2027,13 +2015,13 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>2322</v>
+        <v>5832</v>
       </c>
       <c r="Q17" t="n">
-        <v>114</v>
+        <v>417</v>
       </c>
       <c r="R17" t="n">
-        <v>2436</v>
+        <v>6249</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -2042,12 +2030,12 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1114490806</t>
+          <t>35929022</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1114490806</t>
+          <t>https://m.place.naver.com/place/35929022</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2064,29 +2052,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>일랑헤어 인하본점</t>
+          <t>유니키키헤어</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ilranghair11@naver.com</t>
+          <t>rlrhkd9094@naver.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0507-1429-0212</t>
+          <t>0507-1467-3482</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 인하로 73-1</t>
+          <t>인천광역시 미추홀구 경인로 372 지하1층 B1007호</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ilranghair11</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2096,12 +2084,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2117,17 +2105,17 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>5832</v>
+        <v>462</v>
       </c>
       <c r="Q18" t="n">
-        <v>417</v>
+        <v>18</v>
       </c>
       <c r="R18" t="n">
-        <v>6249</v>
+        <v>480</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -2136,12 +2124,12 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>35929022</t>
+          <t>2065004655</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/35929022</t>
+          <t>https://m.place.naver.com/place/2065004655</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -2158,29 +2146,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>유니키키헤어</t>
+          <t>루엘헤어 시티오씨엘점</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>rlrhkd9094@naver.com</t>
+          <t>ruelhair@naver.com</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0507-1467-3482</t>
+          <t>0507-1447-0543</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 경인로 372 지하1층 B1007호</t>
+          <t>인천광역시 미추홀구 학익로80번길 11 시티오씨엘 3단지 오피스텔상가 3층 311,312호</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/ruelhair_incheon?igsh=cmZmbWw3ZnpjbjFt</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2190,7 +2178,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2211,17 +2199,17 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>462</v>
+        <v>791</v>
       </c>
       <c r="Q19" t="n">
-        <v>18</v>
+        <v>95</v>
       </c>
       <c r="R19" t="n">
-        <v>480</v>
+        <v>886</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2230,12 +2218,12 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2065004655</t>
+          <t>1700200625</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2065004655</t>
+          <t>https://m.place.naver.com/place/1700200625</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -2252,44 +2240,44 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>루엘헤어 시티오씨엘점</t>
+          <t>이철헤어커커 인하대홈플러스점</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ruelhair@naver.com</t>
+          <t>kerker2327@naver.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0507-1447-0543</t>
+          <t>0507-1338-2326</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 학익로80번길 11 시티오씨엘 3단지 오피스텔상가 3층 311,312호</t>
+          <t>인천광역시 미추홀구 소성로 6 홈플러스인하점 지하1층</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/ruelhair_incheon?igsh=cmZmbWw3ZnpjbjFt</t>
+          <t>http://leechulhairkerker.co.kr/</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2300,7 +2288,7 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2309,13 +2297,13 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>791</v>
+        <v>3108</v>
       </c>
       <c r="Q20" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="R20" t="n">
-        <v>886</v>
+        <v>3253</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -2324,12 +2312,12 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1700200625</t>
+          <t>11780793</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1700200625</t>
+          <t>https://m.place.naver.com/place/11780793</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
@@ -2346,39 +2334,39 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>이철헤어커커 인하대홈플러스점</t>
+          <t>헤어더블리 주안본점</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>kerker2327@naver.com</t>
+          <t>hairdoubly_juan@naver.com</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0507-1338-2326</t>
+          <t>0507-1363-9322</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 소성로 6 홈플러스인하점 지하1층</t>
+          <t>인천광역시 미추홀구 미추홀대로 697 유경빌딩 2층</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>http://leechulhairkerker.co.kr/</t>
+          <t>https://blog.naver.com/hairdoubly_juan</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2394,7 +2382,7 @@
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -2403,13 +2391,13 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>3108</v>
+        <v>7490</v>
       </c>
       <c r="Q21" t="n">
-        <v>145</v>
+        <v>1065</v>
       </c>
       <c r="R21" t="n">
-        <v>3253</v>
+        <v>8555</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2418,12 +2406,12 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>11780793</t>
+          <t>1090086912</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/11780793</t>
+          <t>https://m.place.naver.com/place/1090086912</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
@@ -2440,29 +2428,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>헤어더블리 주안본점</t>
+          <t>휴이엠헤어 인천도화점</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>hairdoubly_juan@naver.com</t>
+          <t>vkx0724@naver.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0507-1363-9322</t>
+          <t>0507-1488-7739</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 미추홀대로 697 유경빌딩 2층</t>
+          <t>인천광역시 미추홀구 숙골로 90 도화프라자 203호</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/hairdoubly_juan</t>
+          <t>https://blog.naver.com/vkx0724</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2497,13 +2485,13 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>7490</v>
+        <v>1640</v>
       </c>
       <c r="Q22" t="n">
-        <v>1063</v>
+        <v>49</v>
       </c>
       <c r="R22" t="n">
-        <v>8553</v>
+        <v>1689</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
@@ -2512,12 +2500,12 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1090086912</t>
+          <t>1358473223</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1090086912</t>
+          <t>https://m.place.naver.com/place/1358473223</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
@@ -2534,29 +2522,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>휴이엠헤어 인천도화점</t>
+          <t>테르미니</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>vkx0724@naver.com</t>
+          <t>navely_itsme@naver.com</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0507-1488-7739</t>
+          <t>0507-1486-4435</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 숙골로 90 도화프라자 203호</t>
+          <t>인천광역시 미추홀구 숙골로 93 로데오프라자 203호</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/vkx0724</t>
+          <t>https://www.instagram.com/termini_ggan?igsh=MXhhemd2d2t1ZWtpNQ%3D%3D&amp;utm_source=qr</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2571,7 +2559,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2591,13 +2579,13 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>1640</v>
+        <v>368</v>
       </c>
       <c r="Q23" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="R23" t="n">
-        <v>1689</v>
+        <v>403</v>
       </c>
       <c r="S23" t="inlineStr">
         <is>
@@ -2606,12 +2594,12 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1358473223</t>
+          <t>2061443002</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1358473223</t>
+          <t>https://m.place.naver.com/place/2061443002</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
@@ -2628,29 +2616,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>테르미니</t>
+          <t>이현진헤어프렌즈</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>navely_itsme@naver.com</t>
+          <t>rkdgusrn840321@naver.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0507-1486-4435</t>
+          <t>0507-1482-0927</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 숙골로 93 로데오프라자 203호</t>
+          <t>인천광역시 미추홀구 경원대로 737 1층 이현진헤어프렌즈</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/termini_ggan?igsh=MXhhemd2d2t1ZWtpNQ%3D%3D&amp;utm_source=qr</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2660,7 +2648,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2681,17 +2669,17 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>368</v>
+        <v>346</v>
       </c>
       <c r="Q24" t="n">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="R24" t="n">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="S24" t="inlineStr">
         <is>
@@ -2700,12 +2688,12 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2061443002</t>
+          <t>16491005</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2061443002</t>
+          <t>https://m.place.naver.com/place/16491005</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -2722,29 +2710,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>이현진헤어프렌즈</t>
+          <t>리안헤어 인천미추홀점</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>rkdgusrn840321@naver.com</t>
+          <t>fldks240322@naver.com</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0507-1482-0927</t>
+          <t>0507-1352-2854</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 경원대로 737 1층 이현진헤어프렌즈</t>
+          <t>인천광역시 미추홀구 낙섬중로 129 상가 6동 213호</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/fldks240322</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2754,7 +2742,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2775,17 +2763,17 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P25" t="n">
-        <v>346</v>
+        <v>1469</v>
       </c>
       <c r="Q25" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="R25" t="n">
-        <v>405</v>
+        <v>1529</v>
       </c>
       <c r="S25" t="inlineStr">
         <is>
@@ -2794,12 +2782,12 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>16491005</t>
+          <t>1431476863</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/16491005</t>
+          <t>https://m.place.naver.com/place/1431476863</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
@@ -2816,29 +2804,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>리안헤어 인천미추홀점</t>
+          <t>헤어인숨 용현점</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>fldks240322@naver.com</t>
+          <t>syn77@naver.com</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0507-1352-2854</t>
+          <t>0507-1430-3229</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 낙섬중로 129 상가 6동 213호</t>
+          <t>인천광역시 미추홀구 낙섬동로 134 자이크레스트 근린생활시설동 112호</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fldks240322</t>
+          <t>https://www.instagram.com/h_in_sum?igsh=MWtuOTNyMDhpcWhqMA%3D%3D&amp;utm_source=qr</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2873,13 +2861,13 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>1469</v>
+        <v>268</v>
       </c>
       <c r="Q26" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="R26" t="n">
-        <v>1529</v>
+        <v>290</v>
       </c>
       <c r="S26" t="inlineStr">
         <is>
@@ -2888,12 +2876,12 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1431476863</t>
+          <t>2097295672</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1431476863</t>
+          <t>https://m.place.naver.com/place/2097295672</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
@@ -2910,29 +2898,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>헤어인숨 용현점</t>
+          <t>에프오유헤어 시티오씨엘점</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>syn77@naver.com</t>
+          <t>f5youhair@naver.com</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0507-1430-3229</t>
+          <t>0507-1328-1202</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 낙섬동로 134 자이크레스트 근린생활시설동 112호</t>
+          <t>인천광역시 미추홀구 학익로 116 시티오씨엘1단지 상가 105호 에프오유헤어</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/h_in_sum?igsh=MWtuOTNyMDhpcWhqMA%3D%3D&amp;utm_source=qr</t>
+          <t>https://www.instagram.com/f5you_hair_?igsh=ZXZpdzFpZXR3ZGtz</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2967,13 +2955,13 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="Q27" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="R27" t="n">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="S27" t="inlineStr">
         <is>
@@ -2982,12 +2970,12 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2097295672</t>
+          <t>1443825045</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2097295672</t>
+          <t>https://m.place.naver.com/place/1443825045</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
@@ -3098,29 +3086,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>라비앙르로즈 주안아인애비뉴점</t>
+          <t>헤어위고</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>lavieenrrosejuan@naver.com</t>
+          <t>miffy421m@naver.com</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>032-721-3938</t>
+          <t>0507-1481-7918</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 경인로 372 지하2층 201동</t>
+          <t>인천광역시 미추홀구 염창로 73 상가동 107호 ( 주안동 행복마을아파트 )</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/lavieenr_rose_juan</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3130,7 +3118,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -3151,17 +3139,17 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>4525</v>
+        <v>158</v>
       </c>
       <c r="Q29" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="R29" t="n">
-        <v>4581</v>
+        <v>160</v>
       </c>
       <c r="S29" t="inlineStr">
         <is>
@@ -3170,12 +3158,12 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1095639276</t>
+          <t>1137012839</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1095639276</t>
+          <t>https://m.place.naver.com/place/1137012839</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -3192,34 +3180,34 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>노베르 디 인하</t>
+          <t>라비앙르로즈 주안아인애비뉴점</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>hbs2002i@naver.com</t>
+          <t>lavieenrrosejuan@naver.com</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0507-1304-1527</t>
+          <t>032-721-3938</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 인하로 85 1층</t>
+          <t>인천광역시 미추홀구 경인로 372 지하2층 201동</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://talk.naver.com/profile/c/nanamadehair</t>
+          <t>https://www.instagram.com/lavieenr_rose_juan</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -3234,14 +3222,10 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/profile</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
           <t>X</t>
@@ -3253,13 +3237,13 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>8808</v>
+        <v>4525</v>
       </c>
       <c r="Q30" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="R30" t="n">
-        <v>8843</v>
+        <v>4581</v>
       </c>
       <c r="S30" t="inlineStr">
         <is>
@@ -3268,12 +3252,12 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1177858574</t>
+          <t>1095639276</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1177858574</t>
+          <t>https://m.place.naver.com/place/1095639276</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
@@ -3290,34 +3274,34 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>모드엘헤어 주안아인애비뉴점</t>
+          <t>노베르 디 인하</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>mj_roh34@naver.com</t>
+          <t>hbs2002i@naver.com</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0507-1387-4126</t>
+          <t>0507-1304-1527</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 경인로 372 201동 지하2층 B2102호</t>
+          <t>인천광역시 미추홀구 인하로 85 1층</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mod.l_</t>
+          <t>https://talk.naver.com/profile/c/nanamadehair</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -3332,10 +3316,14 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/profile</t>
+        </is>
+      </c>
       <c r="N31" t="inlineStr">
         <is>
           <t>X</t>
@@ -3347,13 +3335,13 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>103</v>
+        <v>8809</v>
       </c>
       <c r="Q31" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="R31" t="n">
-        <v>110</v>
+        <v>8844</v>
       </c>
       <c r="S31" t="inlineStr">
         <is>
@@ -3362,12 +3350,12 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2055614968</t>
+          <t>1177858574</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2055614968</t>
+          <t>https://m.place.naver.com/place/1177858574</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
@@ -3384,29 +3372,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>26도헤어 인하대역점</t>
+          <t>모드엘헤어 주안아인애비뉴점</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>njms33@naver.com</t>
+          <t>mj_roh34@naver.com</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0507-1400-5987</t>
+          <t>0507-1387-4126</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 용정공원로83번길 49 2층 224호</t>
+          <t>인천광역시 미추홀구 경인로 372 201동 지하2층 B2102호</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/njms33</t>
+          <t>https://www.instagram.com/mod.l_</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3421,7 +3409,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3441,13 +3429,13 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>577</v>
+        <v>103</v>
       </c>
       <c r="Q32" t="n">
-        <v>55</v>
+        <v>7</v>
       </c>
       <c r="R32" t="n">
-        <v>632</v>
+        <v>110</v>
       </c>
       <c r="S32" t="inlineStr">
         <is>
@@ -3456,12 +3444,12 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>2077534385</t>
+          <t>2055614968</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2077534385</t>
+          <t>https://m.place.naver.com/place/2055614968</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
@@ -3478,30 +3466,34 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>붙임머리</t>
+          <t>26도헤어 인하대역점</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>lady_thelady@naver.com</t>
+          <t>njms33@naver.com</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>0507-1400-5987</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 주안중로 28 2층 메종드부티크 인천점</t>
+          <t>인천광역시 미추홀구 용정공원로83번길 49 2층 224호</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://pf.kakao.com/_xoxiCLxd</t>
+          <t>https://blog.naver.com/njms33</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3511,7 +3503,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -3522,7 +3514,7 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -3531,13 +3523,13 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>2395</v>
+        <v>577</v>
       </c>
       <c r="Q33" t="n">
-        <v>674</v>
+        <v>55</v>
       </c>
       <c r="R33" t="n">
-        <v>3069</v>
+        <v>632</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
@@ -3546,12 +3538,12 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1774618150</t>
+          <t>2077534385</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1774618150</t>
+          <t>https://m.place.naver.com/place/2077534385</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
@@ -3568,39 +3560,35 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>엘룩스헤어</t>
+          <t>붙임머리</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>jjhhhhj83@naver.com</t>
+          <t>lady_thelady@naver.com</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>0507-1361-9974</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 주안로 116 리가스퀘어 1층 109호</t>
+          <t>인천광역시 미추홀구 주안중로 28 2층 메종드부티크 인천점</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://pf.kakao.com/_xoxiCLxd</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -3616,22 +3604,22 @@
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>3148</v>
+        <v>2395</v>
       </c>
       <c r="Q34" t="n">
-        <v>311</v>
+        <v>674</v>
       </c>
       <c r="R34" t="n">
-        <v>3459</v>
+        <v>3069</v>
       </c>
       <c r="S34" t="inlineStr">
         <is>
@@ -3640,12 +3628,12 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>31957857</t>
+          <t>1774618150</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/31957857</t>
+          <t>https://m.place.naver.com/place/1774618150</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
@@ -3662,38 +3650,34 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>마하헤어</t>
+          <t>엘룩스헤어</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0163891634@naver.com</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>akh@smartplug.kr</t>
-        </is>
-      </c>
+          <t>jjhhhhj83@naver.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0507-1367-2659</t>
+          <t>0507-1361-9974</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 용정공원로83번길 49 218호2층</t>
+          <t>인천광역시 미추홀구 주안로 116 리가스퀘어 1층 109호</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://booking.naver.com/booking/13/bizes/1137798</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3723,13 +3707,13 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>251</v>
+        <v>3148</v>
       </c>
       <c r="Q35" t="n">
-        <v>3</v>
+        <v>311</v>
       </c>
       <c r="R35" t="n">
-        <v>254</v>
+        <v>3459</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -3738,12 +3722,12 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1307781228</t>
+          <t>31957857</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1307781228</t>
+          <t>https://m.place.naver.com/place/31957857</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -3760,34 +3744,38 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>리안헤어 청운대도화점</t>
+          <t>마하헤어</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>gminish@naver.com</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
+          <t>0163891634@naver.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>akh@smartplug.kr</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>0507-1389-1499</t>
+          <t>0507-1367-2659</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 숙골로 104 와이지프라자 2층 201호</t>
+          <t>인천광역시 미추홀구 용정공원로83번길 49 218호2층</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://booking.naver.com/booking/13/bizes/1137798</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3817,13 +3805,13 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>1372</v>
+        <v>251</v>
       </c>
       <c r="Q36" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="R36" t="n">
-        <v>1387</v>
+        <v>254</v>
       </c>
       <c r="S36" t="inlineStr">
         <is>
@@ -3832,12 +3820,12 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1506960735</t>
+          <t>1307781228</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1506960735</t>
+          <t>https://m.place.naver.com/place/1307781228</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
@@ -3854,29 +3842,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>알팀헤어 용현점</t>
+          <t>리안헤어 청운대도화점</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>kimna0226@naver.com</t>
+          <t>gminish@naver.com</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>0507-1349-9113</t>
+          <t>0507-1389-1499</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 독배로317번길 27 2층 201호 (하남돼지집 건물 2층에 있습니다)</t>
+          <t>인천광역시 미추홀구 숙골로 104 와이지프라자 2층 201호</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/arteam_nayoung</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3886,7 +3874,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3907,17 +3895,17 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>1038</v>
+        <v>1372</v>
       </c>
       <c r="Q37" t="n">
-        <v>377</v>
+        <v>15</v>
       </c>
       <c r="R37" t="n">
-        <v>1415</v>
+        <v>1387</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
@@ -3926,12 +3914,12 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1941487690</t>
+          <t>1506960735</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1941487690</t>
+          <t>https://m.place.naver.com/place/1506960735</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
@@ -3948,29 +3936,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>고정현헤어 앨리웨이인천점</t>
+          <t>알팀헤어 용현점</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>gohair7@naver.com</t>
+          <t>kimna0226@naver.com</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0507-1425-3256</t>
+          <t>0507-1349-9113</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 숙골로87번길 5 234-1, 234-2, 235</t>
+          <t>인천광역시 미추홀구 독배로317번길 27 2층 201호 (하남돼지집 건물 2층에 있습니다)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>http://www.gohair.co.kr</t>
+          <t>https://www.instagram.com/arteam_nayoung</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3985,7 +3973,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -4005,13 +3993,13 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>4372</v>
+        <v>1038</v>
       </c>
       <c r="Q38" t="n">
-        <v>475</v>
+        <v>378</v>
       </c>
       <c r="R38" t="n">
-        <v>4847</v>
+        <v>1416</v>
       </c>
       <c r="S38" t="inlineStr">
         <is>
@@ -4020,12 +4008,12 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1801351487</t>
+          <t>1941487690</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1801351487</t>
+          <t>https://m.place.naver.com/place/1941487690</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
@@ -4042,29 +4030,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>리안헤어 용현점</t>
+          <t>고정현헤어 앨리웨이인천점</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>greenkyj0106@naver.com</t>
+          <t>gohair7@naver.com</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>0507-1415-3013</t>
+          <t>0507-1425-3256</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 토금중로 8 한사랑산부인과 2층</t>
+          <t>인천광역시 미추홀구 숙골로87번길 5 234-1, 234-2, 235</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>http://www.gohair.co.kr</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -4074,12 +4062,12 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -4095,17 +4083,17 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>2351</v>
+        <v>4372</v>
       </c>
       <c r="Q39" t="n">
-        <v>81</v>
+        <v>478</v>
       </c>
       <c r="R39" t="n">
-        <v>2432</v>
+        <v>4850</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
@@ -4114,12 +4102,12 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>43751658</t>
+          <t>1801351487</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/43751658</t>
+          <t>https://m.place.naver.com/place/1801351487</t>
         </is>
       </c>
       <c r="V39" t="inlineStr">
@@ -4131,34 +4119,34 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>남성전문미용실</t>
+          <t>미용실</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>크라운맨즈헤어 주안점</t>
+          <t>리안헤어 용현점</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>crownmensyul@naver.com</t>
+          <t>greenkyj0106@naver.com</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0507-1408-8264</t>
+          <t>0507-1415-3013</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 주안로 107 306호</t>
+          <t>인천광역시 미추홀구 토금중로 8 한사랑산부인과 2층</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/crownmensyul</t>
+          <t>X</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -4168,12 +4156,12 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -4189,17 +4177,17 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>190</v>
+        <v>2351</v>
       </c>
       <c r="Q40" t="n">
-        <v>134</v>
+        <v>81</v>
       </c>
       <c r="R40" t="n">
-        <v>324</v>
+        <v>2432</v>
       </c>
       <c r="S40" t="inlineStr">
         <is>
@@ -4208,12 +4196,12 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>2068984503</t>
+          <t>43751658</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2068984503</t>
+          <t>https://m.place.naver.com/place/43751658</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">
@@ -4225,34 +4213,34 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>미용실</t>
+          <t>남성전문미용실</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>유미주의hair salon</t>
+          <t>크라운맨즈헤어 주안점</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>dbal1040@naver.com</t>
+          <t>crownmensyul@naver.com</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>0507-1354-9136</t>
+          <t>0507-1408-8264</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 용현동 685-12 예승프라자 3층</t>
+          <t>인천광역시 미추홀구 주안로 107 306호</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/estheticism_official</t>
+          <t>https://blog.naver.com/crownmensyul</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -4267,7 +4255,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -4287,13 +4275,13 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>1177</v>
+        <v>191</v>
       </c>
       <c r="Q41" t="n">
-        <v>16</v>
+        <v>134</v>
       </c>
       <c r="R41" t="n">
-        <v>1193</v>
+        <v>325</v>
       </c>
       <c r="S41" t="inlineStr">
         <is>
@@ -4302,12 +4290,12 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1148502864</t>
+          <t>2068984503</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1148502864</t>
+          <t>https://m.place.naver.com/place/2068984503</t>
         </is>
       </c>
       <c r="V41" t="inlineStr">
@@ -4324,29 +4312,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>라벨르봄 도화점</t>
+          <t>유미주의hair salon</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>yijeong0219@naver.com</t>
+          <t>dbal1040@naver.com</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>0507-1394-0665</t>
+          <t>0507-1354-9136</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 숙골로 113 청운대학교 블루클라우드관 B26</t>
+          <t>인천광역시 미추홀구 용현동 685-12 예승프라자 3층</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/labellebom_jane</t>
+          <t>https://www.instagram.com/estheticism_official</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -4381,13 +4369,13 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>3426</v>
+        <v>1177</v>
       </c>
       <c r="Q42" t="n">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="R42" t="n">
-        <v>3488</v>
+        <v>1193</v>
       </c>
       <c r="S42" t="inlineStr">
         <is>
@@ -4396,12 +4384,12 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1877441485</t>
+          <t>1148502864</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1877441485</t>
+          <t>https://m.place.naver.com/place/1148502864</t>
         </is>
       </c>
       <c r="V42" t="inlineStr">
@@ -4418,48 +4406,44 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>루앙뷰티</t>
+          <t>라벨르봄 도화점</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>wkkwkk@naver.com</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>cto@handsos.com</t>
-        </is>
-      </c>
+          <t>yijeong0219@naver.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>0507-1465-2248</t>
+          <t>0507-1394-0665</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 석정로433번길 21 1층</t>
+          <t>인천광역시 미추홀구 숙골로 113 청운대학교 블루클라우드관 B26</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://booking.naver.com/booking/13/bizes/462517</t>
+          <t>https://www.instagram.com/labellebom_jane</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -4479,13 +4463,13 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>604</v>
+        <v>3425</v>
       </c>
       <c r="Q43" t="n">
-        <v>168</v>
+        <v>62</v>
       </c>
       <c r="R43" t="n">
-        <v>772</v>
+        <v>3487</v>
       </c>
       <c r="S43" t="inlineStr">
         <is>
@@ -4494,12 +4478,12 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1636258917</t>
+          <t>1877441485</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1636258917</t>
+          <t>https://m.place.naver.com/place/1877441485</t>
         </is>
       </c>
       <c r="V43" t="inlineStr">
@@ -4516,29 +4500,33 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>드홀헤어 주안점</t>
+          <t>루앙뷰티</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>tngh1357@naver.com</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr"/>
+          <t>wkkwkk@naver.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>cto@handsos.com</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>0507-1364-5869</t>
+          <t>0507-1465-2248</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 인하로 263-1 2층</t>
+          <t>인천광역시 미추홀구 석정로433번길 21 1층</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://talk.naver.com/profile/c/drolehair_juan</t>
+          <t>https://booking.naver.com/booking/13/bizes/462517</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4548,24 +4536,20 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/profile</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
           <t>X</t>
@@ -4573,17 +4557,17 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P44" t="n">
-        <v>3708</v>
+        <v>605</v>
       </c>
       <c r="Q44" t="n">
-        <v>124</v>
+        <v>168</v>
       </c>
       <c r="R44" t="n">
-        <v>3832</v>
+        <v>773</v>
       </c>
       <c r="S44" t="inlineStr">
         <is>
@@ -4592,12 +4576,12 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>1786623547</t>
+          <t>1636258917</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1786623547</t>
+          <t>https://m.place.naver.com/place/1636258917</t>
         </is>
       </c>
       <c r="V44" t="inlineStr">
@@ -4614,34 +4598,30 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>여피헤어</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>yuppiehair@naver.com</t>
-        </is>
-      </c>
+          <t>드홀헤어 주안점</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>0507-1494-4344</t>
+          <t>0507-1364-5869</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 소성로 16 102호</t>
+          <t>인천광역시 미추홀구 인하로 263-1 2층</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/yuppie.hair</t>
+          <t>https://talk.naver.com/profile/c/drolehair_juan</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -4656,10 +4636,14 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr"/>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>https://talk.naver.com/ct/profile</t>
+        </is>
+      </c>
       <c r="N45" t="inlineStr">
         <is>
           <t>X</t>
@@ -4667,17 +4651,17 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P45" t="n">
-        <v>299</v>
+        <v>3708</v>
       </c>
       <c r="Q45" t="n">
-        <v>40</v>
+        <v>124</v>
       </c>
       <c r="R45" t="n">
-        <v>339</v>
+        <v>3832</v>
       </c>
       <c r="S45" t="inlineStr">
         <is>
@@ -4686,12 +4670,12 @@
       </c>
       <c r="T45" t="inlineStr">
         <is>
-          <t>2079885963</t>
+          <t>1786623547</t>
         </is>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2079885963</t>
+          <t>https://m.place.naver.com/place/1786623547</t>
         </is>
       </c>
       <c r="V45" t="inlineStr">
@@ -4708,29 +4692,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>헤어더블리 바이무드 주안점</t>
+          <t>여피헤어</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>qudaktwltb@naver.com</t>
+          <t>yuppiehair@naver.com</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>032-875-9322</t>
+          <t>0507-1494-4344</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 주안로 113 2층 헤어더블리</t>
+          <t>인천광역시 미추홀구 소성로 16 102호</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/qudaktwltb</t>
+          <t>https://www.instagram.com/yuppie.hair</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4745,7 +4729,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -4765,13 +4749,13 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>4383</v>
+        <v>300</v>
       </c>
       <c r="Q46" t="n">
-        <v>766</v>
+        <v>40</v>
       </c>
       <c r="R46" t="n">
-        <v>5149</v>
+        <v>340</v>
       </c>
       <c r="S46" t="inlineStr">
         <is>
@@ -4780,12 +4764,12 @@
       </c>
       <c r="T46" t="inlineStr">
         <is>
-          <t>1554897473</t>
+          <t>2079885963</t>
         </is>
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1554897473</t>
+          <t>https://m.place.naver.com/place/2079885963</t>
         </is>
       </c>
       <c r="V46" t="inlineStr">
@@ -4802,29 +4786,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>먼슬리헤어살롱</t>
+          <t>헤어더블리 바이무드 주안점</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>hyunh485@naver.com</t>
+          <t>qudaktwltb@naver.com</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>0507-1424-0837</t>
+          <t>032-875-9322</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 한나루로 437-1 1층</t>
+          <t>인천광역시 미추홀구 주안로 113 2층 헤어더블리</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/monthly_hair_salon</t>
+          <t>https://blog.naver.com/qudaktwltb</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4839,7 +4823,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -4859,13 +4843,13 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>1472</v>
+        <v>4383</v>
       </c>
       <c r="Q47" t="n">
-        <v>204</v>
+        <v>766</v>
       </c>
       <c r="R47" t="n">
-        <v>1676</v>
+        <v>5149</v>
       </c>
       <c r="S47" t="inlineStr">
         <is>
@@ -4874,12 +4858,12 @@
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>1908912839</t>
+          <t>1554897473</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1908912839</t>
+          <t>https://m.place.naver.com/place/1554897473</t>
         </is>
       </c>
       <c r="V47" t="inlineStr">
@@ -4896,29 +4880,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>로이드밤 인하대역점</t>
+          <t>먼슬리헤어살롱</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>hair3303@naver.com</t>
+          <t>hyunh485@naver.com</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0507-1365-3318</t>
+          <t>0507-1424-0837</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 용정공원로83번길 59 3층 로이드밤인하</t>
+          <t>인천광역시 미추홀구 한나루로 437-1 1층</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/inha_bomb/</t>
+          <t>https://www.instagram.com/monthly_hair_salon</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4953,13 +4937,13 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>6960</v>
+        <v>1472</v>
       </c>
       <c r="Q48" t="n">
-        <v>679</v>
+        <v>205</v>
       </c>
       <c r="R48" t="n">
-        <v>7639</v>
+        <v>1677</v>
       </c>
       <c r="S48" t="inlineStr">
         <is>
@@ -4968,12 +4952,12 @@
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>1414711915</t>
+          <t>1908912839</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1414711915</t>
+          <t>https://m.place.naver.com/place/1908912839</t>
         </is>
       </c>
       <c r="V48" t="inlineStr">
@@ -4990,29 +4974,29 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>에이바헤어 인천주안점</t>
+          <t>로이드밤 인하대역점</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>mpwjdgnsl@naver.com</t>
+          <t>hair3303@naver.com</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0507-1406-9704</t>
+          <t>0507-1365-3318</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 주안로 105-1 1층 일부호</t>
+          <t>인천광역시 미추홀구 용정공원로83번길 59 3층 로이드밤인하</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/seohwi79</t>
+          <t>https://www.instagram.com/inha_bomb/</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -5047,13 +5031,13 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>689</v>
+        <v>6960</v>
       </c>
       <c r="Q49" t="n">
-        <v>206</v>
+        <v>679</v>
       </c>
       <c r="R49" t="n">
-        <v>895</v>
+        <v>7639</v>
       </c>
       <c r="S49" t="inlineStr">
         <is>
@@ -5062,12 +5046,12 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>2042136768</t>
+          <t>1414711915</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2042136768</t>
+          <t>https://m.place.naver.com/place/1414711915</t>
         </is>
       </c>
       <c r="V49" t="inlineStr">
@@ -5084,29 +5068,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>노드온헤어</t>
+          <t>에이바헤어 인천주안점</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>nodehair@naver.com</t>
+          <t>mpwjdgnsl@naver.com</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0507-1374-2383</t>
+          <t>0507-1406-9704</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 용정공원로83번길 49 헤리움 메트로 타워 205호</t>
+          <t>인천광역시 미추홀구 주안로 105-1 1층 일부호</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/nodehair</t>
+          <t>https://www.instagram.com/seohwi79</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -5121,7 +5105,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -5141,13 +5125,13 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>2906</v>
+        <v>689</v>
       </c>
       <c r="Q50" t="n">
-        <v>181</v>
+        <v>206</v>
       </c>
       <c r="R50" t="n">
-        <v>3087</v>
+        <v>895</v>
       </c>
       <c r="S50" t="inlineStr">
         <is>
@@ -5156,12 +5140,12 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>1441530468</t>
+          <t>2042136768</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1441530468</t>
+          <t>https://m.place.naver.com/place/2042136768</t>
         </is>
       </c>
       <c r="V50" t="inlineStr">
@@ -5178,30 +5162,34 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>수다움헤어</t>
+          <t>노드온헤어</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>soodaum1@naver.com</t>
+          <t>nodehair@naver.com</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0507-1374-2383</t>
+        </is>
+      </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 낙섬중로 129 상가5동 121호</t>
+          <t>인천광역시 미추홀구 용정공원로83번길 49 헤리움 메트로 타워 205호</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://link.inpock.co.kr/tndus126</t>
+          <t>https://blog.naver.com/nodehair</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -5222,7 +5210,7 @@
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -5231,13 +5219,13 @@
         </is>
       </c>
       <c r="P51" t="n">
-        <v>121</v>
+        <v>2907</v>
       </c>
       <c r="Q51" t="n">
-        <v>18</v>
+        <v>181</v>
       </c>
       <c r="R51" t="n">
-        <v>139</v>
+        <v>3088</v>
       </c>
       <c r="S51" t="inlineStr">
         <is>
@@ -5246,12 +5234,12 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>2027456892</t>
+          <t>1441530468</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/2027456892</t>
+          <t>https://m.place.naver.com/place/1441530468</t>
         </is>
       </c>
       <c r="V51" t="inlineStr">
@@ -5268,34 +5256,26 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>일랑헤어 주안점</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>ll188l1@naver.com</t>
-        </is>
-      </c>
+          <t>수다움헤어</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>0507-1378-0273</t>
-        </is>
-      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 미추홀대로 729 2층 204호</t>
+          <t>인천광역시 미추홀구 낙섬중로 129 상가5동 121호</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ll188l1</t>
+          <t>https://link.inpock.co.kr/tndus126</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -5316,22 +5296,22 @@
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P52" t="n">
-        <v>2177</v>
+        <v>121</v>
       </c>
       <c r="Q52" t="n">
-        <v>652</v>
+        <v>18</v>
       </c>
       <c r="R52" t="n">
-        <v>2829</v>
+        <v>139</v>
       </c>
       <c r="S52" t="inlineStr">
         <is>
@@ -5340,12 +5320,12 @@
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>1304349290</t>
+          <t>2027456892</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1304349290</t>
+          <t>https://m.place.naver.com/place/2027456892</t>
         </is>
       </c>
       <c r="V52" t="inlineStr">
@@ -5362,29 +5342,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>26도헤어 주안시민공원역점</t>
+          <t>일랑헤어 주안점</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>pinkjump010@naver.com</t>
+          <t>ll188l1@naver.com</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>0507-1334-9389</t>
+          <t>0507-1378-0273</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 미추홀대로 662 2층</t>
+          <t>인천광역시 미추홀구 미추홀대로 729 2층 204호</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/26_hair_jeongmin?igsh=MXNlcGJubXhpc3ZwMw%3D%3D&amp;utm_source=qr</t>
+          <t>https://blog.naver.com/ll188l1</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -5399,7 +5379,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -5415,17 +5395,17 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="P53" t="n">
-        <v>4774</v>
+        <v>2177</v>
       </c>
       <c r="Q53" t="n">
-        <v>82</v>
+        <v>652</v>
       </c>
       <c r="R53" t="n">
-        <v>4856</v>
+        <v>2829</v>
       </c>
       <c r="S53" t="inlineStr">
         <is>
@@ -5434,12 +5414,12 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>1180903010</t>
+          <t>1304349290</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1180903010</t>
+          <t>https://m.place.naver.com/place/1304349290</t>
         </is>
       </c>
       <c r="V53" t="inlineStr">
@@ -5456,29 +5436,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>오프닛헤어 주안시민공원역점</t>
+          <t>26도헤어 주안시민공원역점</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>jyroo728@naver.com</t>
+          <t>syn77@naver.com</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>0507-1334-2159</t>
+          <t>0507-1334-9389</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 인주대로 332 1층 109호</t>
+          <t>인천광역시 미추홀구 미추홀대로 662 2층</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/openit_hair_official</t>
+          <t>https://www.instagram.com/26_hair_jeongmin?igsh=MXNlcGJubXhpc3ZwMw%3D%3D&amp;utm_source=qr</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -5513,13 +5493,13 @@
         </is>
       </c>
       <c r="P54" t="n">
-        <v>2146</v>
+        <v>4774</v>
       </c>
       <c r="Q54" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="R54" t="n">
-        <v>2212</v>
+        <v>4856</v>
       </c>
       <c r="S54" t="inlineStr">
         <is>
@@ -5528,12 +5508,12 @@
       </c>
       <c r="T54" t="inlineStr">
         <is>
-          <t>1726674949</t>
+          <t>1180903010</t>
         </is>
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1726674949</t>
+          <t>https://m.place.naver.com/place/1180903010</t>
         </is>
       </c>
       <c r="V54" t="inlineStr">
@@ -5550,29 +5530,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>에리카헤어 용현점</t>
+          <t>오프닛헤어 주안시민공원역점</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>elica5875@naver.com</t>
+          <t>jyroo728@naver.com</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>0507-1326-5875</t>
+          <t>0507-1334-2159</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 낙섬중로 61 2층</t>
+          <t>인천광역시 미추홀구 인주대로 332 1층 109호</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/elica5875</t>
+          <t>https://www.instagram.com/openit_hair_official</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -5587,7 +5567,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -5607,13 +5587,13 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>3409</v>
+        <v>2147</v>
       </c>
       <c r="Q55" t="n">
-        <v>277</v>
+        <v>66</v>
       </c>
       <c r="R55" t="n">
-        <v>3686</v>
+        <v>2213</v>
       </c>
       <c r="S55" t="inlineStr">
         <is>
@@ -5622,12 +5602,12 @@
       </c>
       <c r="T55" t="inlineStr">
         <is>
-          <t>1171114652</t>
+          <t>1726674949</t>
         </is>
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1171114652</t>
+          <t>https://m.place.naver.com/place/1726674949</t>
         </is>
       </c>
       <c r="V55" t="inlineStr">
@@ -5639,39 +5619,39 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>남성전문미용실</t>
+          <t>미용실</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>노바 맨즈헤어 본점</t>
+          <t>에리카헤어 용현점</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>qwqw634@naver.com</t>
+          <t>elica5875@naver.com</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>0507-1436-1690</t>
+          <t>0507-1326-5875</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 인하로 87 1층</t>
+          <t>인천광역시 미추홀구 낙섬중로 61 2층</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>http://젠틀엠헤어인하대.kr</t>
+          <t>https://blog.naver.com/elica5875</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -5681,7 +5661,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -5701,13 +5681,13 @@
         </is>
       </c>
       <c r="P56" t="n">
-        <v>356</v>
+        <v>3409</v>
       </c>
       <c r="Q56" t="n">
-        <v>7</v>
+        <v>277</v>
       </c>
       <c r="R56" t="n">
-        <v>363</v>
+        <v>3686</v>
       </c>
       <c r="S56" t="inlineStr">
         <is>
@@ -5716,12 +5696,12 @@
       </c>
       <c r="T56" t="inlineStr">
         <is>
-          <t>1629040441</t>
+          <t>1171114652</t>
         </is>
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1629040441</t>
+          <t>https://m.place.naver.com/place/1171114652</t>
         </is>
       </c>
       <c r="V56" t="inlineStr">
@@ -5733,39 +5713,35 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>미용실</t>
+          <t>남성전문미용실</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>일랑헤어 2호점</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>ilranghair1@naver.com</t>
-        </is>
-      </c>
+          <t>노바 맨즈헤어 본점</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>032-876-0212</t>
+          <t>0507-1436-1690</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 인하로77번길 37 2층</t>
+          <t>인천광역시 미추홀구 인하로 87 1층</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/ilranghair1</t>
+          <t>http://젠틀엠헤어인하대.kr</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -5775,7 +5751,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -5791,17 +5767,17 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P57" t="n">
-        <v>5201</v>
+        <v>356</v>
       </c>
       <c r="Q57" t="n">
-        <v>297</v>
+        <v>7</v>
       </c>
       <c r="R57" t="n">
-        <v>5498</v>
+        <v>363</v>
       </c>
       <c r="S57" t="inlineStr">
         <is>
@@ -5810,12 +5786,12 @@
       </c>
       <c r="T57" t="inlineStr">
         <is>
-          <t>1374136455</t>
+          <t>1629040441</t>
         </is>
       </c>
       <c r="U57" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1374136455</t>
+          <t>https://m.place.naver.com/place/1629040441</t>
         </is>
       </c>
       <c r="V57" t="inlineStr">
@@ -5832,29 +5808,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>디온헤어</t>
+          <t>일랑헤어 2호점</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>dion1703@naver.com</t>
+          <t>ilranghair1@naver.com</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>0507-1449-3557</t>
+          <t>032-876-0212</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>인천광역시 미추홀구 숙골로 114 1층 108호 디온헤어</t>
+          <t>인천광역시 미추홀구 인하로77번길 37 2층</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://youtube.com/shorts/fQLlCD_n798?feature=shared</t>
+          <t>https://blog.naver.com/ilranghair1</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5869,7 +5845,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -5889,13 +5865,13 @@
         </is>
       </c>
       <c r="P58" t="n">
-        <v>269</v>
+        <v>5201</v>
       </c>
       <c r="Q58" t="n">
-        <v>27</v>
+        <v>297</v>
       </c>
       <c r="R58" t="n">
-        <v>296</v>
+        <v>5498</v>
       </c>
       <c r="S58" t="inlineStr">
         <is>
@@ -5904,12 +5880,12 @@
       </c>
       <c r="T58" t="inlineStr">
         <is>
-          <t>1852587066</t>
+          <t>1374136455</t>
         </is>
       </c>
       <c r="U58" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1852587066</t>
+          <t>https://m.place.naver.com/place/1374136455</t>
         </is>
       </c>
       <c r="V58" t="inlineStr">
@@ -6399,11 +6375,7 @@
           <t>에이바헤어 신기사거리점</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>iii_9@naver.com</t>
-        </is>
-      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
@@ -6641,13 +6613,13 @@
         </is>
       </c>
       <c r="P66" t="n">
-        <v>6773</v>
+        <v>6777</v>
       </c>
       <c r="Q66" t="n">
         <v>1380</v>
       </c>
       <c r="R66" t="n">
-        <v>8153</v>
+        <v>8157</v>
       </c>
       <c r="S66" t="inlineStr">
         <is>
@@ -7016,10 +6988,10 @@
         <v>4772</v>
       </c>
       <c r="Q70" t="n">
-        <v>747</v>
+        <v>753</v>
       </c>
       <c r="R70" t="n">
-        <v>5519</v>
+        <v>5525</v>
       </c>
       <c r="S70" t="inlineStr">
         <is>
@@ -7149,7 +7121,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>qwd563@naver.com</t>
+          <t>wow9493@naver.com</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>

</xml_diff>